<commit_message>
Harden production academic submission package
</commit_message>
<xml_diff>
--- a/results/dynamic_mechanism_ranking/exports/dynamic_mechanism_results.xlsx
+++ b/results/dynamic_mechanism_ranking/exports/dynamic_mechanism_results.xlsx
@@ -76,7 +76,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-19T20:31:28.974334+00:00</t>
+          <t>2026-06-23T11:56:25.416948+00:00</t>
         </is>
       </c>
     </row>
@@ -88,7 +88,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-19T20:28:11.635225+00:00</t>
+          <t>2026-06-23T11:55:28.946025+00:00</t>
         </is>
       </c>
     </row>
@@ -197,7 +197,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>0.175078468060665</v>
+        <v>0.271723506555857</v>
       </c>
     </row>
     <row r="14">
@@ -208,7 +208,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>configs/graphs/macro_modules.yaml macro-module proxy graph; not a subject structural connectome</t>
+          <t>mean positive placebo FC proxy graph; not a structural connectome</t>
         </is>
       </c>
     </row>
@@ -390,22 +390,22 @@
         <v>4</v>
       </c>
       <c r="D2">
-        <v>16.9155969309102</v>
+        <v>14.7053387389715</v>
       </c>
       <c r="E2">
-        <v>13.0351997808519</v>
+        <v>11.5278433807344</v>
       </c>
       <c r="F2">
-        <v>-46.6908029835861</v>
+        <v>-23.871455842959</v>
       </c>
       <c r="G2">
-        <v>-27.2062778020286</v>
+        <v>-7.32946763512973</v>
       </c>
       <c r="H2">
-        <v>-321.300465644201</v>
+        <v>-95.9848586856354</v>
       </c>
       <c r="I2">
-        <v>-675.759055875662</v>
+        <v>-187.963682489796</v>
       </c>
       <c r="J2">
         <v>0.160179830246317</v>
@@ -426,22 +426,22 @@
         <v>4</v>
       </c>
       <c r="D3">
-        <v>15.033358447397</v>
+        <v>13.1396751682226</v>
       </c>
       <c r="E3">
-        <v>10.1263886845241</v>
+        <v>8.64526911536635</v>
       </c>
       <c r="F3">
-        <v>-80.8171086631551</v>
+        <v>-55.3851145751782</v>
       </c>
       <c r="G3">
-        <v>-48.6878482068684</v>
+        <v>-34.1257651188264</v>
       </c>
       <c r="H3">
-        <v>-467.899477404191</v>
+        <v>-173.270211468708</v>
       </c>
       <c r="I3">
-        <v>-1039.11576706904</v>
+        <v>-184.907644076059</v>
       </c>
       <c r="J3">
         <v>-0.315915604205742</v>
@@ -462,22 +462,22 @@
         <v>4</v>
       </c>
       <c r="D4">
-        <v>26.1282407044397</v>
+        <v>25.4563236831059</v>
       </c>
       <c r="E4">
-        <v>24.3856460318154</v>
+        <v>22.6808203955743</v>
       </c>
       <c r="F4">
-        <v>-51.7472751091316</v>
+        <v>-32.6119316121857</v>
       </c>
       <c r="G4">
-        <v>-35.711127695522</v>
+        <v>-19.1870653230731</v>
       </c>
       <c r="H4">
-        <v>-295.405723540866</v>
+        <v>-85.4357034348274</v>
       </c>
       <c r="I4">
-        <v>-643.646524757176</v>
+        <v>-155.949380358173</v>
       </c>
       <c r="J4">
         <v>0.333014394158394</v>
@@ -498,22 +498,22 @@
         <v>4</v>
       </c>
       <c r="D5">
-        <v>17.9717831649739</v>
+        <v>12.9882313541631</v>
       </c>
       <c r="E5">
-        <v>17.5437543202525</v>
+        <v>12.1091179232483</v>
       </c>
       <c r="F5">
-        <v>-46.817008124183</v>
+        <v>-25.0568982488129</v>
       </c>
       <c r="G5">
-        <v>-18.1066482578109</v>
+        <v>-1.99541474410424</v>
       </c>
       <c r="H5">
-        <v>-310.153164859368</v>
+        <v>-114.473532185919</v>
       </c>
       <c r="I5">
-        <v>-790.371957100348</v>
+        <v>-193.728245509087</v>
       </c>
       <c r="J5">
         <v>0.354849941297024</v>
@@ -534,22 +534,22 @@
         <v>4</v>
       </c>
       <c r="D6">
-        <v>11.0545181278768</v>
+        <v>10.3803404407038</v>
       </c>
       <c r="E6">
-        <v>9.30218709761174</v>
+        <v>9.46769246770156</v>
       </c>
       <c r="F6">
-        <v>-8.26666748606205</v>
+        <v>2.06037366897296</v>
       </c>
       <c r="G6">
-        <v>5.84397493388227</v>
+        <v>15.0366503012331</v>
       </c>
       <c r="H6">
-        <v>-206.15224898246</v>
+        <v>-108.464423613763</v>
       </c>
       <c r="I6">
-        <v>-446.047739391572</v>
+        <v>-162.301068517883</v>
       </c>
       <c r="J6">
         <v>0.507089830745447</v>
@@ -570,22 +570,22 @@
         <v>4</v>
       </c>
       <c r="D7">
-        <v>-2.99637359429998</v>
+        <v>-8.26631393544112</v>
       </c>
       <c r="E7">
-        <v>-2.19251192412966</v>
+        <v>-6.72255257936693</v>
       </c>
       <c r="F7">
-        <v>-35.1911617352854</v>
+        <v>-8.63000210445936</v>
       </c>
       <c r="G7">
-        <v>-17.2907371891958</v>
+        <v>5.26983134357545</v>
       </c>
       <c r="H7">
-        <v>-244.723629387244</v>
+        <v>-71.0792470017014</v>
       </c>
       <c r="I7">
-        <v>-584.569018472162</v>
+        <v>-142.891350273477</v>
       </c>
       <c r="J7">
         <v>-0.423893635398318</v>
@@ -606,22 +606,22 @@
         <v>4</v>
       </c>
       <c r="D8">
-        <v>-2.85037739562286</v>
+        <v>-5.06173611315342</v>
       </c>
       <c r="E8">
-        <v>4.3349094315384</v>
+        <v>2.0865792174385</v>
       </c>
       <c r="F8">
-        <v>-3.64802548585194</v>
+        <v>-5.65157297984831</v>
       </c>
       <c r="G8">
-        <v>8.0033412484283</v>
+        <v>11.3698360176128</v>
       </c>
       <c r="H8">
-        <v>-65.4695632714699</v>
+        <v>-15.529787316433</v>
       </c>
       <c r="I8">
-        <v>-219.386535206372</v>
+        <v>-414.798040218961</v>
       </c>
       <c r="J8">
         <v>-0.0741156429112876</v>
@@ -642,22 +642,22 @@
         <v>4</v>
       </c>
       <c r="D9">
-        <v>-5.32263652949888</v>
+        <v>-5.84944148313472</v>
       </c>
       <c r="E9">
-        <v>1.4554442634252</v>
+        <v>2.31984911907579</v>
       </c>
       <c r="F9">
-        <v>-29.0148069917065</v>
+        <v>-14.0323934264265</v>
       </c>
       <c r="G9">
-        <v>-14.8903037060932</v>
+        <v>0.664118108100063</v>
       </c>
       <c r="H9">
-        <v>-198.207980615454</v>
+        <v>-59.6062767915889</v>
       </c>
       <c r="I9">
-        <v>-382.490949666448</v>
+        <v>-117.393847935845</v>
       </c>
       <c r="J9">
         <v>0.198183039205768</v>
@@ -678,22 +678,22 @@
         <v>4</v>
       </c>
       <c r="D10">
-        <v>-12.8881959824675</v>
+        <v>-15.9878121115851</v>
       </c>
       <c r="E10">
-        <v>-4.15863547937574</v>
+        <v>-5.36052226476569</v>
       </c>
       <c r="F10">
-        <v>-7.90876191148551</v>
+        <v>-9.25670519377843</v>
       </c>
       <c r="G10">
-        <v>6.32698608442069</v>
+        <v>7.5195865862839</v>
       </c>
       <c r="H10">
-        <v>-421.661302008998</v>
+        <v>-302.284421660907</v>
       </c>
       <c r="I10">
-        <v>-703.689412454525</v>
+        <v>-562.287946447247</v>
       </c>
       <c r="J10">
         <v>-0.266484518065128</v>
@@ -714,22 +714,22 @@
         <v>4</v>
       </c>
       <c r="D11">
-        <v>-7.70092151213217</v>
+        <v>-11.7887634819232</v>
       </c>
       <c r="E11">
-        <v>-1.81020906806011</v>
+        <v>-3.98023384778894</v>
       </c>
       <c r="F11">
-        <v>-14.4220479827361</v>
+        <v>-18.5416836463397</v>
       </c>
       <c r="G11">
-        <v>2.68192215673474</v>
+        <v>3.13189615883969</v>
       </c>
       <c r="H11">
-        <v>-592.778590374237</v>
+        <v>-391.473157652103</v>
       </c>
       <c r="I11">
-        <v>-908.383660928582</v>
+        <v>-710.361744343501</v>
       </c>
       <c r="J11">
         <v>-0.069962491412073</v>
@@ -750,22 +750,22 @@
         <v>4</v>
       </c>
       <c r="D12">
-        <v>-20.1536952245376</v>
+        <v>-23.07241854873</v>
       </c>
       <c r="E12">
-        <v>-11.5982658684941</v>
+        <v>-12.4747558729671</v>
       </c>
       <c r="F12">
-        <v>-20.9241802688133</v>
+        <v>-9.85468368639787</v>
       </c>
       <c r="G12">
-        <v>2.46237818705736</v>
+        <v>12.6576232399184</v>
       </c>
       <c r="H12">
-        <v>-470.821188277758</v>
+        <v>-357.613491730543</v>
       </c>
       <c r="I12">
-        <v>-911.924729543908</v>
+        <v>-541.520443642531</v>
       </c>
       <c r="J12">
         <v>0.402691656263688</v>
@@ -786,22 +786,22 @@
         <v>4</v>
       </c>
       <c r="D13">
-        <v>-10.0138954292664</v>
+        <v>-10.9247870714693</v>
       </c>
       <c r="E13">
-        <v>-1.18001072742519</v>
+        <v>-1.84562351919374</v>
       </c>
       <c r="F13">
-        <v>-75.9802318841546</v>
+        <v>-54.3604895814566</v>
       </c>
       <c r="G13">
-        <v>-40.2108597874049</v>
+        <v>-21.4928632630995</v>
       </c>
       <c r="H13">
-        <v>-574.913478027509</v>
+        <v>-269.835845957458</v>
       </c>
       <c r="I13">
-        <v>-1505.57778562035</v>
+        <v>-780.816451121795</v>
       </c>
       <c r="J13">
         <v>0.312987748181705</v>
@@ -822,22 +822,22 @@
         <v>4</v>
       </c>
       <c r="D14">
-        <v>11.0605688576467</v>
+        <v>6.92942643417413</v>
       </c>
       <c r="E14">
-        <v>12.865694098794</v>
+        <v>8.50962238740043</v>
       </c>
       <c r="F14">
-        <v>-0.287000481055065</v>
+        <v>4.01960967667809</v>
       </c>
       <c r="G14">
-        <v>11.1416505009983</v>
+        <v>17.7867394015449</v>
       </c>
       <c r="H14">
-        <v>-170.930469916843</v>
+        <v>-88.0643004253058</v>
       </c>
       <c r="I14">
-        <v>-335.702939743926</v>
+        <v>-257.487503245238</v>
       </c>
       <c r="J14">
         <v>0.35379213051035</v>
@@ -858,22 +858,22 @@
         <v>4</v>
       </c>
       <c r="D15">
-        <v>15.9543806106084</v>
+        <v>18.2302512479764</v>
       </c>
       <c r="E15">
-        <v>14.1589026871813</v>
+        <v>14.3830588459216</v>
       </c>
       <c r="F15">
-        <v>-25.3151992859835</v>
+        <v>-11.5136024170293</v>
       </c>
       <c r="G15">
-        <v>-11.0708562080111</v>
+        <v>3.19675993612621</v>
       </c>
       <c r="H15">
-        <v>-231.659793082335</v>
+        <v>-82.1628413269725</v>
       </c>
       <c r="I15">
-        <v>-452.672753507222</v>
+        <v>-198.88523403213</v>
       </c>
       <c r="J15">
         <v>0.0246121349070163</v>
@@ -894,22 +894,22 @@
         <v>4</v>
       </c>
       <c r="D16">
-        <v>5.98546924470024</v>
+        <v>3.783379294446</v>
       </c>
       <c r="E16">
-        <v>1.95360665672545</v>
+        <v>0.812813592203181</v>
       </c>
       <c r="F16">
-        <v>-82.4719135156976</v>
+        <v>-58.5871063688691</v>
       </c>
       <c r="G16">
-        <v>-50.2822454024228</v>
+        <v>-38.0572582713317</v>
       </c>
       <c r="H16">
-        <v>-473.683209666616</v>
+        <v>-226.448264229073</v>
       </c>
       <c r="I16">
-        <v>-1299.7453463658</v>
+        <v>-459.45268711086</v>
       </c>
       <c r="J16">
         <v>-0.0509858204342158</v>
@@ -930,22 +930,22 @@
         <v>4</v>
       </c>
       <c r="D17">
-        <v>6.5236105564922</v>
+        <v>4.80698621004573</v>
       </c>
       <c r="E17">
-        <v>3.27720349445639</v>
+        <v>1.55578156119915</v>
       </c>
       <c r="F17">
-        <v>-74.9862592329402</v>
+        <v>-52.2940898338739</v>
       </c>
       <c r="G17">
-        <v>-44.2665795351665</v>
+        <v>-28.0094798851265</v>
       </c>
       <c r="H17">
-        <v>-454.976859840197</v>
+        <v>-234.453405673611</v>
       </c>
       <c r="I17">
-        <v>-1032.14454393015</v>
+        <v>-390.63695432147</v>
       </c>
       <c r="J17">
         <v>-0.29458957589458</v>
@@ -966,22 +966,22 @@
         <v>4</v>
       </c>
       <c r="D18">
-        <v>6.29971068193502</v>
+        <v>-0.440805178585179</v>
       </c>
       <c r="E18">
-        <v>11.090214749392</v>
+        <v>5.5480714199708</v>
       </c>
       <c r="F18">
-        <v>-26.4081500260642</v>
+        <v>-11.4446869661343</v>
       </c>
       <c r="G18">
-        <v>-12.409581254238</v>
+        <v>0.733599440565422</v>
       </c>
       <c r="H18">
-        <v>-207.13374583405</v>
+        <v>-64.3816578713939</v>
       </c>
       <c r="I18">
-        <v>-442.260457626078</v>
+        <v>-130.570350517664</v>
       </c>
       <c r="J18">
         <v>0.496348121058154</v>
@@ -1002,22 +1002,22 @@
         <v>4</v>
       </c>
       <c r="D19">
-        <v>16.0071512238274</v>
+        <v>13.2876067640025</v>
       </c>
       <c r="E19">
-        <v>11.3755202060343</v>
+        <v>9.65435965454938</v>
       </c>
       <c r="F19">
-        <v>-27.7266889335177</v>
+        <v>-12.6385701625299</v>
       </c>
       <c r="G19">
-        <v>-10.0829238923441</v>
+        <v>1.17287529974033</v>
       </c>
       <c r="H19">
-        <v>-253.124358023514</v>
+        <v>-102.488941109286</v>
       </c>
       <c r="I19">
-        <v>-555.106053384923</v>
+        <v>-156.699354408055</v>
       </c>
       <c r="J19">
         <v>-0.435780295010088</v>
@@ -1038,22 +1038,22 @@
         <v>4</v>
       </c>
       <c r="D20">
-        <v>6.29027921324869</v>
+        <v>10.2327505758782</v>
       </c>
       <c r="E20">
-        <v>5.18266853866057</v>
+        <v>7.96104829516897</v>
       </c>
       <c r="F20">
-        <v>-51.2518378511199</v>
+        <v>-31.3986137224325</v>
       </c>
       <c r="G20">
-        <v>-28.0534462827341</v>
+        <v>-12.6947760490282</v>
       </c>
       <c r="H20">
-        <v>-366.401932383604</v>
+        <v>-161.226837912763</v>
       </c>
       <c r="I20">
-        <v>-851.995764015938</v>
+        <v>-235.977995308521</v>
       </c>
       <c r="J20">
         <v>0.288787466883299</v>
@@ -1074,22 +1074,22 @@
         <v>4</v>
       </c>
       <c r="D21">
-        <v>0.0514838241929241</v>
+        <v>2.05982038067396</v>
       </c>
       <c r="E21">
-        <v>5.5861129784703</v>
+        <v>7.80771528690873</v>
       </c>
       <c r="F21">
-        <v>-15.6264752607012</v>
+        <v>2.7329536149284</v>
       </c>
       <c r="G21">
-        <v>0.609012548836766</v>
+        <v>14.3689032756522</v>
       </c>
       <c r="H21">
-        <v>-155.826223878245</v>
+        <v>-26.3682220518872</v>
       </c>
       <c r="I21">
-        <v>-556.541189963181</v>
+        <v>-50.9166149127535</v>
       </c>
       <c r="J21">
         <v>0.235886724780995</v>
@@ -1110,22 +1110,22 @@
         <v>4</v>
       </c>
       <c r="D22">
-        <v>-8.86010578507523</v>
+        <v>-14.9901725869463</v>
       </c>
       <c r="E22">
-        <v>4.07111231334483</v>
+        <v>0.435571210436502</v>
       </c>
       <c r="F22">
-        <v>-20.0925725452399</v>
+        <v>-14.9684915348496</v>
       </c>
       <c r="G22">
-        <v>-7.07087984614403</v>
+        <v>1.1990434624587</v>
       </c>
       <c r="H22">
-        <v>-224.241024820978</v>
+        <v>-137.223944128137</v>
       </c>
       <c r="I22">
-        <v>-380.722621563015</v>
+        <v>-431.640815060434</v>
       </c>
       <c r="J22">
         <v>0.108218070185883</v>
@@ -1146,22 +1146,22 @@
         <v>4</v>
       </c>
       <c r="D23">
-        <v>2.79189209147252</v>
+        <v>-0.383616168141245</v>
       </c>
       <c r="E23">
-        <v>11.8624132978669</v>
+        <v>9.49533306799054</v>
       </c>
       <c r="F23">
-        <v>-11.0600634505696</v>
+        <v>1.1270369478368</v>
       </c>
       <c r="G23">
-        <v>0.578261891685436</v>
+        <v>13.6310451032443</v>
       </c>
       <c r="H23">
-        <v>-211.565419876526</v>
+        <v>-101.672276097644</v>
       </c>
       <c r="I23">
-        <v>-372.233948748234</v>
+        <v>-172.156664675344</v>
       </c>
       <c r="J23">
         <v>0.218273482225619</v>
@@ -1182,22 +1182,22 @@
         <v>4</v>
       </c>
       <c r="D24">
-        <v>19.2986962738389</v>
+        <v>16.8262500841253</v>
       </c>
       <c r="E24">
-        <v>19.1426073561923</v>
+        <v>16.1991880560293</v>
       </c>
       <c r="F24">
-        <v>-34.235690820572</v>
+        <v>-12.7699115987839</v>
       </c>
       <c r="G24">
-        <v>-18.3470810759041</v>
+        <v>-1.08568242104221</v>
       </c>
       <c r="H24">
-        <v>-238.485983930779</v>
+        <v>-72.1575776834375</v>
       </c>
       <c r="I24">
-        <v>-562.641062669187</v>
+        <v>-93.5677299121642</v>
       </c>
       <c r="J24">
         <v>0.580424329458897</v>
@@ -1218,22 +1218,22 @@
         <v>4</v>
       </c>
       <c r="D25">
-        <v>24.9593599753844</v>
+        <v>23.1806439548001</v>
       </c>
       <c r="E25">
-        <v>25.0974482188169</v>
+        <v>22.0091561572407</v>
       </c>
       <c r="F25">
-        <v>-23.0454227013007</v>
+        <v>-4.01907305995886</v>
       </c>
       <c r="G25">
-        <v>-9.62578747316995</v>
+        <v>7.51715800784476</v>
       </c>
       <c r="H25">
-        <v>-211.553986337598</v>
+        <v>-70.1567355520224</v>
       </c>
       <c r="I25">
-        <v>-440.96404153203</v>
+        <v>-92.0644311122696</v>
       </c>
       <c r="J25">
         <v>0.304275523540752</v>
@@ -1254,22 +1254,22 @@
         <v>4</v>
       </c>
       <c r="D26">
-        <v>0.820610304506136</v>
+        <v>-0.368342896543898</v>
       </c>
       <c r="E26">
-        <v>0.681618652078876</v>
+        <v>-0.290388286880913</v>
       </c>
       <c r="F26">
-        <v>-55.5976675806168</v>
+        <v>-28.0929186083813</v>
       </c>
       <c r="G26">
-        <v>-25.9975309891832</v>
+        <v>-6.38779077420265</v>
       </c>
       <c r="H26">
-        <v>-430.300354598075</v>
+        <v>-215.612479112461</v>
       </c>
       <c r="I26">
-        <v>-1279.64525428361</v>
+        <v>-564.328579215826</v>
       </c>
       <c r="J26">
         <v>0.313938142940463</v>
@@ -1290,22 +1290,22 @@
         <v>4</v>
       </c>
       <c r="D27">
-        <v>-8.76951892399488</v>
+        <v>-7.61196494447154</v>
       </c>
       <c r="E27">
-        <v>-9.03552513758554</v>
+        <v>-7.21069404955123</v>
       </c>
       <c r="F27">
-        <v>-55.30315702903</v>
+        <v>-22.7929227587823</v>
       </c>
       <c r="G27">
-        <v>-30.8464639805607</v>
+        <v>-8.30287489116626</v>
       </c>
       <c r="H27">
-        <v>-324.987265446136</v>
+        <v>-89.2402566306559</v>
       </c>
       <c r="I27">
-        <v>-1035.12876770101</v>
+        <v>-257.638566239757</v>
       </c>
       <c r="J27">
         <v>-0.0465586385533015</v>
@@ -1326,22 +1326,22 @@
         <v>4</v>
       </c>
       <c r="D28">
-        <v>27.0960030122215</v>
+        <v>23.3556299096288</v>
       </c>
       <c r="E28">
-        <v>25.7751043709151</v>
+        <v>21.2922536013703</v>
       </c>
       <c r="F28">
-        <v>-28.8968199548251</v>
+        <v>-11.7812471024027</v>
       </c>
       <c r="G28">
-        <v>-13.9360798878152</v>
+        <v>1.31901991523678</v>
       </c>
       <c r="H28">
-        <v>-215.145214901087</v>
+        <v>-66.7645894104906</v>
       </c>
       <c r="I28">
-        <v>-362.340070944581</v>
+        <v>-160.049145213662</v>
       </c>
       <c r="J28">
         <v>0.184954437802717</v>
@@ -1362,22 +1362,22 @@
         <v>4</v>
       </c>
       <c r="D29">
-        <v>-6.73960337672682</v>
+        <v>-10.8514796343557</v>
       </c>
       <c r="E29">
-        <v>0.109048485501237</v>
+        <v>-3.72937104131617</v>
       </c>
       <c r="F29">
-        <v>-42.1105173141508</v>
+        <v>-15.4915399599841</v>
       </c>
       <c r="G29">
-        <v>-19.0372474490151</v>
+        <v>2.05965187525534</v>
       </c>
       <c r="H29">
-        <v>-285.831150842683</v>
+        <v>-96.7050050163799</v>
       </c>
       <c r="I29">
-        <v>-790.735895173455</v>
+        <v>-191.006275511487</v>
       </c>
       <c r="J29">
         <v>0.568160129311668</v>
@@ -1398,22 +1398,22 @@
         <v>4</v>
       </c>
       <c r="D30">
-        <v>3.72444117836127</v>
+        <v>-1.34752245478102</v>
       </c>
       <c r="E30">
-        <v>7.94113441521863</v>
+        <v>3.70307694446837</v>
       </c>
       <c r="F30">
-        <v>-31.1909415272388</v>
+        <v>-21.2394444662337</v>
       </c>
       <c r="G30">
-        <v>-13.6838489060317</v>
+        <v>-3.70575326848372</v>
       </c>
       <c r="H30">
-        <v>-216.178317536675</v>
+        <v>-98.8702153690552</v>
       </c>
       <c r="I30">
-        <v>-367.78475708017</v>
+        <v>-280.225731263221</v>
       </c>
       <c r="J30">
         <v>0.00933423778054267</v>
@@ -1434,22 +1434,22 @@
         <v>4</v>
       </c>
       <c r="D31">
-        <v>-6.60587547440534</v>
+        <v>-8.42268186752115</v>
       </c>
       <c r="E31">
-        <v>-2.30199934826197</v>
+        <v>-4.45657269947354</v>
       </c>
       <c r="F31">
-        <v>-4.57519798843815</v>
+        <v>-9.30181458070148</v>
       </c>
       <c r="G31">
-        <v>6.68830625272919</v>
+        <v>8.41246140745993</v>
       </c>
       <c r="H31">
-        <v>-172.574768137007</v>
+        <v>-113.22179028219</v>
       </c>
       <c r="I31">
-        <v>-300.150824897307</v>
+        <v>-376.4287524802</v>
       </c>
       <c r="J31">
         <v>0.0123793711666004</v>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>0.821660429963266</v>
+        <v>0.77798078426263</v>
       </c>
       <c r="E2">
         <v>4</v>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D3">
-        <v>1.2053002825115</v>
+        <v>0.963696123644589</v>
       </c>
       <c r="E3">
         <v>4</v>
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="D4">
-        <v>3.46165921744938</v>
+        <v>1.52472454063851</v>
       </c>
       <c r="E4">
         <v>4</v>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
       <c r="D5">
-        <v>3.43777448908647</v>
+        <v>3.0641890476422</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="D6">
-        <v>6.37410519398694</v>
+        <v>2.24030211542567</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="D7">
-        <v>1.29284221254488</v>
+        <v>1.16943438192814</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="D8">
-        <v>0.851359517056847</v>
+        <v>0.81194980329452</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="D9">
-        <v>0.947516351659399</v>
+        <v>0.897885869443337</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="D10">
-        <v>0.800288896475404</v>
+        <v>0.688938024383754</v>
       </c>
       <c r="E10">
         <v>4</v>
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="D11">
-        <v>1.4470592435591</v>
+        <v>1.07050713854067</v>
       </c>
       <c r="E11">
         <v>4</v>
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="D12">
-        <v>4.54483646080759</v>
+        <v>1.88266239612182</v>
       </c>
       <c r="E12">
         <v>4</v>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="D13">
-        <v>1.94251249072694</v>
+        <v>2.48992030655298</v>
       </c>
       <c r="E13">
         <v>4</v>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="D14">
-        <v>9.11621700185414</v>
+        <v>1.9628370944159</v>
       </c>
       <c r="E14">
         <v>4</v>
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D15">
-        <v>1.84043045248676</v>
+        <v>1.55253885567053</v>
       </c>
       <c r="E15">
         <v>4</v>
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="D16">
-        <v>0.875842389731378</v>
+        <v>0.636239433596116</v>
       </c>
       <c r="E16">
         <v>4</v>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="D17">
-        <v>0.973219574437457</v>
+        <v>0.798136836417871</v>
       </c>
       <c r="E17">
         <v>4</v>
@@ -1874,7 +1874,7 @@
         </is>
       </c>
       <c r="D18">
-        <v>0.636232394863204</v>
+        <v>0.567334110897721</v>
       </c>
       <c r="E18">
         <v>4</v>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="D19">
-        <v>0.965465322566483</v>
+        <v>0.752352723156288</v>
       </c>
       <c r="E19">
         <v>4</v>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
       <c r="D20">
-        <v>2.51569930431023</v>
+        <v>1.05203999936891</v>
       </c>
       <c r="E20">
         <v>4</v>
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="D21">
-        <v>1.74520279491066</v>
+        <v>1.47107492340725</v>
       </c>
       <c r="E21">
         <v>4</v>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="D22">
-        <v>4.73132009377957</v>
+        <v>1.45208814140327</v>
       </c>
       <c r="E22">
         <v>4</v>
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="D23">
-        <v>0.730039361553513</v>
+        <v>0.70121215403635</v>
       </c>
       <c r="E23">
         <v>4</v>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="D24">
-        <v>0.619867022509525</v>
+        <v>0.514079670797377</v>
       </c>
       <c r="E24">
         <v>4</v>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="D25">
-        <v>0.711412055120916</v>
+        <v>0.631236888933318</v>
       </c>
       <c r="E25">
         <v>4</v>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="D26">
-        <v>1.14124455509859</v>
+        <v>1.04095494387707</v>
       </c>
       <c r="E26">
         <v>4</v>
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D27">
-        <v>1.67554111117589</v>
+        <v>1.30178596498033</v>
       </c>
       <c r="E27">
         <v>4</v>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="D28">
-        <v>4.68085066152207</v>
+        <v>2.2325728365971</v>
       </c>
       <c r="E28">
         <v>4</v>
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="D29">
-        <v>6.81980339931521</v>
+        <v>5.09869783393697</v>
       </c>
       <c r="E29">
         <v>4</v>
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="D30">
-        <v>10.1613214805324</v>
+        <v>3.05757869319022</v>
       </c>
       <c r="E30">
         <v>4</v>
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D31">
-        <v>3.74210349073613</v>
+        <v>3.59088552519127</v>
       </c>
       <c r="E31">
         <v>4</v>
@@ -2196,7 +2196,7 @@
         </is>
       </c>
       <c r="D32">
-        <v>1.42636667221659</v>
+        <v>1.25943951658184</v>
       </c>
       <c r="E32">
         <v>4</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="D33">
-        <v>1.41866790387482</v>
+        <v>1.27631812493373</v>
       </c>
       <c r="E33">
         <v>4</v>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="D34">
-        <v>0.648141775514433</v>
+        <v>0.655900294379105</v>
       </c>
       <c r="E34">
         <v>4</v>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
       <c r="D35">
-        <v>0.701721500934469</v>
+        <v>0.642386297419002</v>
       </c>
       <c r="E35">
         <v>4</v>
@@ -2288,7 +2288,7 @@
         </is>
       </c>
       <c r="D36">
-        <v>1.98430062233228</v>
+        <v>1.36731876815837</v>
       </c>
       <c r="E36">
         <v>4</v>
@@ -2311,7 +2311,7 @@
         </is>
       </c>
       <c r="D37">
-        <v>3.57560202427309</v>
+        <v>1.35012277670495</v>
       </c>
       <c r="E37">
         <v>4</v>
@@ -2334,7 +2334,7 @@
         </is>
       </c>
       <c r="D38">
-        <v>3.53916351324896</v>
+        <v>1.72043348056833</v>
       </c>
       <c r="E38">
         <v>4</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="D39">
-        <v>0.637433475811075</v>
+        <v>1.06338652805112</v>
       </c>
       <c r="E39">
         <v>4</v>
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="D40">
-        <v>0.633024539279238</v>
+        <v>0.654223968978531</v>
       </c>
       <c r="E40">
         <v>4</v>
@@ -2403,7 +2403,7 @@
         </is>
       </c>
       <c r="D41">
-        <v>0.745275196612973</v>
+        <v>0.756074589451274</v>
       </c>
       <c r="E41">
         <v>4</v>
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="D42">
-        <v>0.544572941464497</v>
+        <v>0.512788739427027</v>
       </c>
       <c r="E42">
         <v>4</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D43">
-        <v>0.736214486061869</v>
+        <v>0.55704241843101</v>
       </c>
       <c r="E43">
         <v>4</v>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="D44">
-        <v>1.87727160847729</v>
+        <v>0.877275114121274</v>
       </c>
       <c r="E44">
         <v>4</v>
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="D45">
-        <v>2.97051148876281</v>
+        <v>1.30577165990535</v>
       </c>
       <c r="E45">
         <v>4</v>
@@ -2518,7 +2518,7 @@
         </is>
       </c>
       <c r="D46">
-        <v>3.72797764024849</v>
+        <v>1.24551949324465</v>
       </c>
       <c r="E46">
         <v>4</v>
@@ -2541,7 +2541,7 @@
         </is>
       </c>
       <c r="D47">
-        <v>0.504557141660284</v>
+        <v>0.634138626099557</v>
       </c>
       <c r="E47">
         <v>4</v>
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="D48">
-        <v>0.562337353614656</v>
+        <v>0.576226651625461</v>
       </c>
       <c r="E48">
         <v>4</v>
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D49">
-        <v>0.627683399136897</v>
+        <v>0.588030641485859</v>
       </c>
       <c r="E49">
         <v>4</v>
@@ -2610,7 +2610,7 @@
         </is>
       </c>
       <c r="D50">
-        <v>0.484690139926066</v>
+        <v>0.598875617236304</v>
       </c>
       <c r="E50">
         <v>4</v>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="D51">
-        <v>0.50237175975798</v>
+        <v>0.632721509802931</v>
       </c>
       <c r="E51">
         <v>4</v>
@@ -2656,7 +2656,7 @@
         </is>
       </c>
       <c r="D52">
-        <v>0.802014657755537</v>
+        <v>0.691879726883077</v>
       </c>
       <c r="E52">
         <v>4</v>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="D53">
-        <v>2.44906952391535</v>
+        <v>2.10817843198488</v>
       </c>
       <c r="E53">
         <v>4</v>
@@ -2702,7 +2702,7 @@
         </is>
       </c>
       <c r="D54">
-        <v>1.54803504439678</v>
+        <v>3.0829999408817</v>
       </c>
       <c r="E54">
         <v>4</v>
@@ -2725,7 +2725,7 @@
         </is>
       </c>
       <c r="D55">
-        <v>0.586062761677501</v>
+        <v>0.82845894309987</v>
       </c>
       <c r="E55">
         <v>4</v>
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="D56">
-        <v>0.476791305114119</v>
+        <v>0.697469216753557</v>
       </c>
       <c r="E56">
         <v>4</v>
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D57">
-        <v>0.546076092953101</v>
+        <v>0.713889584959661</v>
       </c>
       <c r="E57">
         <v>4</v>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="D58">
-        <v>0.474571858636465</v>
+        <v>0.459197494248713</v>
       </c>
       <c r="E58">
         <v>4</v>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="D59">
-        <v>0.612267967456789</v>
+        <v>0.523633893245984</v>
       </c>
       <c r="E59">
         <v>4</v>
@@ -2840,7 +2840,7 @@
         </is>
       </c>
       <c r="D60">
-        <v>1.41521115620903</v>
+        <v>0.732908023690641</v>
       </c>
       <c r="E60">
         <v>4</v>
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="D61">
-        <v>2.40862204299956</v>
+        <v>1.12120698614488</v>
       </c>
       <c r="E61">
         <v>4</v>
@@ -2886,7 +2886,7 @@
         </is>
       </c>
       <c r="D62">
-        <v>2.28976626758479</v>
+        <v>0.998267102372257</v>
       </c>
       <c r="E62">
         <v>4</v>
@@ -2909,7 +2909,7 @@
         </is>
       </c>
       <c r="D63">
-        <v>0.516049367958413</v>
+        <v>0.598923637133546</v>
       </c>
       <c r="E63">
         <v>4</v>
@@ -2932,7 +2932,7 @@
         </is>
       </c>
       <c r="D64">
-        <v>0.462253206907341</v>
+        <v>0.443992831875145</v>
       </c>
       <c r="E64">
         <v>4</v>
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="D65">
-        <v>0.532915265872273</v>
+        <v>0.52713469017753</v>
       </c>
       <c r="E65">
         <v>4</v>
@@ -2978,7 +2978,7 @@
         </is>
       </c>
       <c r="D66">
-        <v>0.638336072155148</v>
+        <v>0.759210081458875</v>
       </c>
       <c r="E66">
         <v>4</v>
@@ -3001,7 +3001,7 @@
         </is>
       </c>
       <c r="D67">
-        <v>0.688820552297027</v>
+        <v>0.829487920500969</v>
       </c>
       <c r="E67">
         <v>4</v>
@@ -3024,7 +3024,7 @@
         </is>
       </c>
       <c r="D68">
-        <v>3.32995226519764</v>
+        <v>3.05418388538814</v>
       </c>
       <c r="E68">
         <v>4</v>
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="D69">
-        <v>2.75074290541571</v>
+        <v>2.14825876150182</v>
       </c>
       <c r="E69">
         <v>4</v>
@@ -3070,7 +3070,7 @@
         </is>
       </c>
       <c r="D70">
-        <v>5.130239427789</v>
+        <v>5.02815685771446</v>
       </c>
       <c r="E70">
         <v>4</v>
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="D71">
-        <v>0.98747557588279</v>
+        <v>1.43467351834707</v>
       </c>
       <c r="E71">
         <v>4</v>
@@ -3116,7 +3116,7 @@
         </is>
       </c>
       <c r="D72">
-        <v>0.651644385188199</v>
+        <v>0.850567165117943</v>
       </c>
       <c r="E72">
         <v>4</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="D73">
-        <v>0.735345777299118</v>
+        <v>0.896933620733517</v>
       </c>
       <c r="E73">
         <v>4</v>
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="D74">
-        <v>0.702105001700354</v>
+        <v>0.891758675083982</v>
       </c>
       <c r="E74">
         <v>4</v>
@@ -3185,7 +3185,7 @@
         </is>
       </c>
       <c r="D75">
-        <v>0.803362921934769</v>
+        <v>1.05710574750684</v>
       </c>
       <c r="E75">
         <v>4</v>
@@ -3208,7 +3208,7 @@
         </is>
       </c>
       <c r="D76">
-        <v>4.86403313372672</v>
+        <v>4.3827545190718</v>
       </c>
       <c r="E76">
         <v>4</v>
@@ -3231,7 +3231,7 @@
         </is>
       </c>
       <c r="D77">
-        <v>2.88930209454851</v>
+        <v>2.21529852810772</v>
       </c>
       <c r="E77">
         <v>4</v>
@@ -3254,7 +3254,7 @@
         </is>
       </c>
       <c r="D78">
-        <v>7.07991211970871</v>
+        <v>7.22647115474505</v>
       </c>
       <c r="E78">
         <v>4</v>
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="D79">
-        <v>1.55024496345756</v>
+        <v>2.10311522459931</v>
       </c>
       <c r="E79">
         <v>4</v>
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="D80">
-        <v>0.73796440567694</v>
+        <v>1.00272185514741</v>
       </c>
       <c r="E80">
         <v>4</v>
@@ -3323,7 +3323,7 @@
         </is>
       </c>
       <c r="D81">
-        <v>0.825502249673096</v>
+        <v>1.09128361719585</v>
       </c>
       <c r="E81">
         <v>4</v>
@@ -3346,7 +3346,7 @@
         </is>
       </c>
       <c r="D82">
-        <v>0.476775278893432</v>
+        <v>0.468703406280701</v>
       </c>
       <c r="E82">
         <v>4</v>
@@ -3369,7 +3369,7 @@
         </is>
       </c>
       <c r="D83">
-        <v>0.576536597726231</v>
+        <v>0.514892644397036</v>
       </c>
       <c r="E83">
         <v>4</v>
@@ -3392,7 +3392,7 @@
         </is>
       </c>
       <c r="D84">
-        <v>2.72153431239409</v>
+        <v>2.14485002334111</v>
       </c>
       <c r="E84">
         <v>4</v>
@@ -3415,7 +3415,7 @@
         </is>
       </c>
       <c r="D85">
-        <v>3.2454862216968</v>
+        <v>3.34101299196036</v>
       </c>
       <c r="E85">
         <v>4</v>
@@ -3438,7 +3438,7 @@
         </is>
       </c>
       <c r="D86">
-        <v>4.82460695147458</v>
+        <v>3.00682817133961</v>
       </c>
       <c r="E86">
         <v>4</v>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="D87">
-        <v>1.78143516882024</v>
+        <v>1.78115607640025</v>
       </c>
       <c r="E87">
         <v>4</v>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="D88">
-        <v>0.536319593826408</v>
+        <v>0.493544957392874</v>
       </c>
       <c r="E88">
         <v>4</v>
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="D89">
-        <v>0.591091506036421</v>
+        <v>0.589510685988521</v>
       </c>
       <c r="E89">
         <v>4</v>
@@ -3530,7 +3530,7 @@
         </is>
       </c>
       <c r="D90">
-        <v>1.80194646292565</v>
+        <v>2.02812407634074</v>
       </c>
       <c r="E90">
         <v>4</v>
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D91">
-        <v>3.17106956388488</v>
+        <v>3.13062225355897</v>
       </c>
       <c r="E91">
         <v>4</v>
@@ -3576,7 +3576,7 @@
         </is>
       </c>
       <c r="D92">
-        <v>12.1615795451252</v>
+        <v>7.50072983480166</v>
       </c>
       <c r="E92">
         <v>4</v>
@@ -3599,7 +3599,7 @@
         </is>
       </c>
       <c r="D93">
-        <v>5.30179571131244</v>
+        <v>4.66988311940485</v>
       </c>
       <c r="E93">
         <v>4</v>
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="D94">
-        <v>28.9316521175058</v>
+        <v>17.8640505135712</v>
       </c>
       <c r="E94">
         <v>4</v>
@@ -3645,7 +3645,7 @@
         </is>
       </c>
       <c r="D95">
-        <v>7.34706009791982</v>
+        <v>7.23074719121909</v>
       </c>
       <c r="E95">
         <v>4</v>
@@ -3668,7 +3668,7 @@
         </is>
       </c>
       <c r="D96">
-        <v>2.14075874020217</v>
+        <v>2.11798133569711</v>
       </c>
       <c r="E96">
         <v>4</v>
@@ -3691,7 +3691,7 @@
         </is>
       </c>
       <c r="D97">
-        <v>2.26164333397072</v>
+        <v>2.57679518736786</v>
       </c>
       <c r="E97">
         <v>4</v>
@@ -3714,7 +3714,7 @@
         </is>
       </c>
       <c r="D98">
-        <v>0.633975497855789</v>
+        <v>0.719559937314379</v>
       </c>
       <c r="E98">
         <v>4</v>
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D99">
-        <v>0.635795010584406</v>
+        <v>0.690636436444592</v>
       </c>
       <c r="E99">
         <v>4</v>
@@ -3760,7 +3760,7 @@
         </is>
       </c>
       <c r="D100">
-        <v>1.71763279549833</v>
+        <v>1.35323536225106</v>
       </c>
       <c r="E100">
         <v>4</v>
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="D101">
-        <v>3.69543318576467</v>
+        <v>3.70718139903014</v>
       </c>
       <c r="E101">
         <v>4</v>
@@ -3806,7 +3806,7 @@
         </is>
       </c>
       <c r="D102">
-        <v>2.76224988141386</v>
+        <v>2.57233685425817</v>
       </c>
       <c r="E102">
         <v>4</v>
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D103">
-        <v>0.866416039143066</v>
+        <v>1.0374600385016</v>
       </c>
       <c r="E103">
         <v>4</v>
@@ -3852,7 +3852,7 @@
         </is>
       </c>
       <c r="D104">
-        <v>0.685667299203105</v>
+        <v>0.909502923434393</v>
       </c>
       <c r="E104">
         <v>4</v>
@@ -3875,7 +3875,7 @@
         </is>
       </c>
       <c r="D105">
-        <v>0.715515215136366</v>
+        <v>0.840054793371825</v>
       </c>
       <c r="E105">
         <v>4</v>
@@ -3898,7 +3898,7 @@
         </is>
       </c>
       <c r="D106">
-        <v>0.545239252684941</v>
+        <v>0.563256530353056</v>
       </c>
       <c r="E106">
         <v>4</v>
@@ -3921,7 +3921,7 @@
         </is>
       </c>
       <c r="D107">
-        <v>0.683267656087541</v>
+        <v>0.628107647845861</v>
       </c>
       <c r="E107">
         <v>4</v>
@@ -3944,7 +3944,7 @@
         </is>
       </c>
       <c r="D108">
-        <v>1.80833937725855</v>
+        <v>1.02604409965085</v>
       </c>
       <c r="E108">
         <v>4</v>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="D109">
-        <v>2.67877339909498</v>
+        <v>2.63854897210184</v>
       </c>
       <c r="E109">
         <v>4</v>
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="D110">
-        <v>3.01338879101606</v>
+        <v>1.68349059894699</v>
       </c>
       <c r="E110">
         <v>4</v>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="D111">
-        <v>0.732640935336713</v>
+        <v>0.759044402855608</v>
       </c>
       <c r="E111">
         <v>4</v>
@@ -4036,7 +4036,7 @@
         </is>
       </c>
       <c r="D112">
-        <v>0.518868808003058</v>
+        <v>0.569148672313851</v>
       </c>
       <c r="E112">
         <v>4</v>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="D113">
-        <v>0.615163760696984</v>
+        <v>0.648849818902152</v>
       </c>
       <c r="E113">
         <v>4</v>
@@ -4082,7 +4082,7 @@
         </is>
       </c>
       <c r="D114">
-        <v>0.735746098364201</v>
+        <v>0.526447431526792</v>
       </c>
       <c r="E114">
         <v>4</v>
@@ -4105,7 +4105,7 @@
         </is>
       </c>
       <c r="D115">
-        <v>1.34252998430224</v>
+        <v>0.834877748211573</v>
       </c>
       <c r="E115">
         <v>4</v>
@@ -4128,7 +4128,7 @@
         </is>
       </c>
       <c r="D116">
-        <v>4.22085183209265</v>
+        <v>1.71857850229775</v>
       </c>
       <c r="E116">
         <v>4</v>
@@ -4151,7 +4151,7 @@
         </is>
       </c>
       <c r="D117">
-        <v>4.38685287135875</v>
+        <v>2.22251361026174</v>
       </c>
       <c r="E117">
         <v>4</v>
@@ -4174,7 +4174,7 @@
         </is>
       </c>
       <c r="D118">
-        <v>10.2985717729208</v>
+        <v>2.94522430190274</v>
       </c>
       <c r="E118">
         <v>4</v>
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="D119">
-        <v>1.19546353807318</v>
+        <v>0.965672201724866</v>
       </c>
       <c r="E119">
         <v>4</v>
@@ -4220,7 +4220,7 @@
         </is>
       </c>
       <c r="D120">
-        <v>0.702398408415003</v>
+        <v>0.417163534405391</v>
       </c>
       <c r="E120">
         <v>4</v>
@@ -4243,7 +4243,7 @@
         </is>
       </c>
       <c r="D121">
-        <v>0.893339050602581</v>
+        <v>0.604732962732565</v>
       </c>
       <c r="E121">
         <v>4</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="D122">
-        <v>0.839311106417086</v>
+        <v>0.677248943987065</v>
       </c>
       <c r="E122">
         <v>4</v>
@@ -4289,7 +4289,7 @@
         </is>
       </c>
       <c r="D123">
-        <v>1.46867910844586</v>
+        <v>1.03141011515462</v>
       </c>
       <c r="E123">
         <v>4</v>
@@ -4312,7 +4312,7 @@
         </is>
       </c>
       <c r="D124">
-        <v>4.65798242268356</v>
+        <v>2.26508215805331</v>
       </c>
       <c r="E124">
         <v>4</v>
@@ -4335,7 +4335,7 @@
         </is>
       </c>
       <c r="D125">
-        <v>5.478480036971</v>
+        <v>3.53058106838631</v>
       </c>
       <c r="E125">
         <v>4</v>
@@ -4358,7 +4358,7 @@
         </is>
       </c>
       <c r="D126">
-        <v>9.50221489790083</v>
+        <v>3.32283359195245</v>
       </c>
       <c r="E126">
         <v>4</v>
@@ -4381,7 +4381,7 @@
         </is>
       </c>
       <c r="D127">
-        <v>2.05019651614019</v>
+        <v>1.95855727036328</v>
       </c>
       <c r="E127">
         <v>4</v>
@@ -4404,7 +4404,7 @@
         </is>
       </c>
       <c r="D128">
-        <v>0.903871609905791</v>
+        <v>0.66565791848261</v>
       </c>
       <c r="E128">
         <v>4</v>
@@ -4427,7 +4427,7 @@
         </is>
       </c>
       <c r="D129">
-        <v>1.01803142015151</v>
+        <v>0.805729478848124</v>
       </c>
       <c r="E129">
         <v>4</v>
@@ -4450,7 +4450,7 @@
         </is>
       </c>
       <c r="D130">
-        <v>0.603805302552473</v>
+        <v>0.595099379438629</v>
       </c>
       <c r="E130">
         <v>4</v>
@@ -4473,7 +4473,7 @@
         </is>
       </c>
       <c r="D131">
-        <v>0.763259112715861</v>
+        <v>0.663206640552788</v>
       </c>
       <c r="E131">
         <v>4</v>
@@ -4496,7 +4496,7 @@
         </is>
       </c>
       <c r="D132">
-        <v>1.85448984327403</v>
+        <v>0.978234225903595</v>
       </c>
       <c r="E132">
         <v>4</v>
@@ -4519,7 +4519,7 @@
         </is>
       </c>
       <c r="D133">
-        <v>2.09423534091813</v>
+        <v>0.987462451793603</v>
       </c>
       <c r="E133">
         <v>4</v>
@@ -4542,7 +4542,7 @@
         </is>
       </c>
       <c r="D134">
-        <v>3.27419739679156</v>
+        <v>1.37212272510009</v>
       </c>
       <c r="E134">
         <v>4</v>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="D135">
-        <v>0.441535179311146</v>
+        <v>0.600353312180634</v>
       </c>
       <c r="E135">
         <v>4</v>
@@ -4588,7 +4588,7 @@
         </is>
       </c>
       <c r="D136">
-        <v>0.582340879648799</v>
+        <v>0.583332226778</v>
       </c>
       <c r="E136">
         <v>4</v>
@@ -4611,7 +4611,7 @@
         </is>
       </c>
       <c r="D137">
-        <v>0.678998270609682</v>
+        <v>0.668107876194927</v>
       </c>
       <c r="E137">
         <v>4</v>
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="D138">
-        <v>0.650738285620805</v>
+        <v>0.589684016173317</v>
       </c>
       <c r="E138">
         <v>4</v>
@@ -4657,7 +4657,7 @@
         </is>
       </c>
       <c r="D139">
-        <v>0.831166465846191</v>
+        <v>0.664211644294606</v>
       </c>
       <c r="E139">
         <v>4</v>
@@ -4680,7 +4680,7 @@
         </is>
       </c>
       <c r="D140">
-        <v>2.29791539351168</v>
+        <v>1.19404492024006</v>
       </c>
       <c r="E140">
         <v>4</v>
@@ -4703,7 +4703,7 @@
         </is>
       </c>
       <c r="D141">
-        <v>3.25457544762507</v>
+        <v>1.85382364898497</v>
       </c>
       <c r="E141">
         <v>4</v>
@@ -4726,7 +4726,7 @@
         </is>
       </c>
       <c r="D142">
-        <v>4.26302590079516</v>
+        <v>1.5137150625644</v>
       </c>
       <c r="E142">
         <v>4</v>
@@ -4749,7 +4749,7 @@
         </is>
       </c>
       <c r="D143">
-        <v>0.905661857935477</v>
+        <v>1.00020042789002</v>
       </c>
       <c r="E143">
         <v>4</v>
@@ -4772,7 +4772,7 @@
         </is>
       </c>
       <c r="D144">
-        <v>0.650173005471369</v>
+        <v>0.566461404564199</v>
       </c>
       <c r="E144">
         <v>4</v>
@@ -4795,7 +4795,7 @@
         </is>
       </c>
       <c r="D145">
-        <v>0.75503669093949</v>
+        <v>0.672094474375475</v>
       </c>
       <c r="E145">
         <v>4</v>
@@ -4818,7 +4818,7 @@
         </is>
       </c>
       <c r="D146">
-        <v>0.597361076373317</v>
+        <v>0.501293106198336</v>
       </c>
       <c r="E146">
         <v>4</v>
@@ -4841,7 +4841,7 @@
         </is>
       </c>
       <c r="D147">
-        <v>0.903519606621873</v>
+        <v>0.658692192230735</v>
       </c>
       <c r="E147">
         <v>4</v>
@@ -4864,7 +4864,7 @@
         </is>
       </c>
       <c r="D148">
-        <v>2.78610360351265</v>
+        <v>1.30951212999658</v>
       </c>
       <c r="E148">
         <v>4</v>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D149">
-        <v>3.01947799571515</v>
+        <v>2.07495565227537</v>
       </c>
       <c r="E149">
         <v>4</v>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="D150">
-        <v>5.68685214295398</v>
+        <v>1.68423452882498</v>
       </c>
       <c r="E150">
         <v>4</v>
@@ -4933,7 +4933,7 @@
         </is>
       </c>
       <c r="D151">
-        <v>1.30737553981101</v>
+        <v>1.12410182773835</v>
       </c>
       <c r="E151">
         <v>4</v>
@@ -4956,7 +4956,7 @@
         </is>
       </c>
       <c r="D152">
-        <v>0.630258158168694</v>
+        <v>0.463326474198048</v>
       </c>
       <c r="E152">
         <v>4</v>
@@ -4979,7 +4979,7 @@
         </is>
       </c>
       <c r="D153">
-        <v>0.70558007835803</v>
+        <v>0.584492214567399</v>
       </c>
       <c r="E153">
         <v>4</v>
@@ -5002,7 +5002,7 @@
         </is>
       </c>
       <c r="D154">
-        <v>0.525246905308985</v>
+        <v>0.504696418407402</v>
       </c>
       <c r="E154">
         <v>4</v>
@@ -5025,7 +5025,7 @@
         </is>
       </c>
       <c r="D155">
-        <v>0.607324483024693</v>
+        <v>0.490903299396122</v>
       </c>
       <c r="E155">
         <v>4</v>
@@ -5048,7 +5048,7 @@
         </is>
       </c>
       <c r="D156">
-        <v>1.34371932388932</v>
+        <v>0.637775890700987</v>
       </c>
       <c r="E156">
         <v>4</v>
@@ -5071,7 +5071,7 @@
         </is>
       </c>
       <c r="D157">
-        <v>3.338828508959</v>
+        <v>1.70071875632553</v>
       </c>
       <c r="E157">
         <v>4</v>
@@ -5094,7 +5094,7 @@
         </is>
       </c>
       <c r="D158">
-        <v>3.4484622823604</v>
+        <v>0.761670750246357</v>
       </c>
       <c r="E158">
         <v>4</v>
@@ -5117,7 +5117,7 @@
         </is>
       </c>
       <c r="D159">
-        <v>0.56537184739053</v>
+        <v>0.648186882136071</v>
       </c>
       <c r="E159">
         <v>4</v>
@@ -5140,7 +5140,7 @@
         </is>
       </c>
       <c r="D160">
-        <v>0.519878128884547</v>
+        <v>0.529541367327683</v>
       </c>
       <c r="E160">
         <v>4</v>
@@ -5163,7 +5163,7 @@
         </is>
       </c>
       <c r="D161">
-        <v>0.611045828801236</v>
+        <v>0.573276903104923</v>
       </c>
       <c r="E161">
         <v>4</v>
@@ -5186,7 +5186,7 @@
         </is>
       </c>
       <c r="D162">
-        <v>0.630347363900482</v>
+        <v>0.735047425786847</v>
       </c>
       <c r="E162">
         <v>4</v>
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="D163">
-        <v>0.757000365279193</v>
+        <v>0.845072937492881</v>
       </c>
       <c r="E163">
         <v>4</v>
@@ -5232,7 +5232,7 @@
         </is>
       </c>
       <c r="D164">
-        <v>2.04384475264294</v>
+        <v>1.7437084946639</v>
       </c>
       <c r="E164">
         <v>4</v>
@@ -5255,7 +5255,7 @@
         </is>
       </c>
       <c r="D165">
-        <v>2.56065857619862</v>
+        <v>2.30273565054048</v>
       </c>
       <c r="E165">
         <v>4</v>
@@ -5278,7 +5278,7 @@
         </is>
       </c>
       <c r="D166">
-        <v>3.03022237269575</v>
+        <v>3.90781212553393</v>
       </c>
       <c r="E166">
         <v>4</v>
@@ -5301,7 +5301,7 @@
         </is>
       </c>
       <c r="D167">
-        <v>0.683600258371108</v>
+        <v>1.01830709536259</v>
       </c>
       <c r="E167">
         <v>4</v>
@@ -5324,7 +5324,7 @@
         </is>
       </c>
       <c r="D168">
-        <v>0.609965581958902</v>
+        <v>0.78705243718176</v>
       </c>
       <c r="E168">
         <v>4</v>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="D169">
-        <v>0.707008634249544</v>
+        <v>0.855328700357045</v>
       </c>
       <c r="E169">
         <v>4</v>
@@ -5370,7 +5370,7 @@
         </is>
       </c>
       <c r="D170">
-        <v>0.698426080892106</v>
+        <v>0.752154420685931</v>
       </c>
       <c r="E170">
         <v>4</v>
@@ -5393,7 +5393,7 @@
         </is>
       </c>
       <c r="D171">
-        <v>0.7756724485941</v>
+        <v>0.743677362460013</v>
       </c>
       <c r="E171">
         <v>4</v>
@@ -5416,7 +5416,7 @@
         </is>
       </c>
       <c r="D172">
-        <v>2.17605415145865</v>
+        <v>1.51688693996636</v>
       </c>
       <c r="E172">
         <v>4</v>
@@ -5439,7 +5439,7 @@
         </is>
       </c>
       <c r="D173">
-        <v>3.18644632748108</v>
+        <v>1.69476509800901</v>
       </c>
       <c r="E173">
         <v>4</v>
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D174">
-        <v>3.29820506088433</v>
+        <v>2.04703838454699</v>
       </c>
       <c r="E174">
         <v>4</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="D175">
-        <v>0.528014353332263</v>
+        <v>0.909483043992635</v>
       </c>
       <c r="E175">
         <v>4</v>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="D176">
-        <v>0.704737105429633</v>
+        <v>0.842841301306618</v>
       </c>
       <c r="E176">
         <v>4</v>
@@ -5531,7 +5531,7 @@
         </is>
       </c>
       <c r="D177">
-        <v>0.780183955091438</v>
+        <v>0.861047078025889</v>
       </c>
       <c r="E177">
         <v>4</v>
@@ -5554,7 +5554,7 @@
         </is>
       </c>
       <c r="D178">
-        <v>0.603314973669326</v>
+        <v>0.562162047103986</v>
       </c>
       <c r="E178">
         <v>4</v>
@@ -5577,7 +5577,7 @@
         </is>
       </c>
       <c r="D179">
-        <v>0.809864022728972</v>
+        <v>0.633949643561079</v>
       </c>
       <c r="E179">
         <v>4</v>
@@ -5600,7 +5600,7 @@
         </is>
       </c>
       <c r="D180">
-        <v>2.04213662482634</v>
+        <v>0.967804562949847</v>
       </c>
       <c r="E180">
         <v>4</v>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="D181">
-        <v>2.30952118912094</v>
+        <v>1.14655866071932</v>
       </c>
       <c r="E181">
         <v>4</v>
@@ -5646,7 +5646,7 @@
         </is>
       </c>
       <c r="D182">
-        <v>3.99781275276475</v>
+        <v>1.08816431300694</v>
       </c>
       <c r="E182">
         <v>4</v>
@@ -5669,7 +5669,7 @@
         </is>
       </c>
       <c r="D183">
-        <v>0.471361775565119</v>
+        <v>0.634964378240413</v>
       </c>
       <c r="E183">
         <v>4</v>
@@ -5692,7 +5692,7 @@
         </is>
       </c>
       <c r="D184">
-        <v>0.585407958889362</v>
+        <v>0.537424738331947</v>
       </c>
       <c r="E184">
         <v>4</v>
@@ -5715,7 +5715,7 @@
         </is>
       </c>
       <c r="D185">
-        <v>0.684312629738245</v>
+        <v>0.627140885215129</v>
       </c>
       <c r="E185">
         <v>4</v>
@@ -5738,7 +5738,7 @@
         </is>
       </c>
       <c r="D186">
-        <v>0.747088169068621</v>
+        <v>0.74843661362627</v>
       </c>
       <c r="E186">
         <v>4</v>
@@ -5761,7 +5761,7 @@
         </is>
       </c>
       <c r="D187">
-        <v>0.919257795581893</v>
+        <v>0.778516827935392</v>
       </c>
       <c r="E187">
         <v>4</v>
@@ -5784,7 +5784,7 @@
         </is>
       </c>
       <c r="D188">
-        <v>2.32758297218986</v>
+        <v>1.27351530942256</v>
       </c>
       <c r="E188">
         <v>4</v>
@@ -5807,7 +5807,7 @@
         </is>
       </c>
       <c r="D189">
-        <v>3.2316981546755</v>
+        <v>1.81346070398956</v>
       </c>
       <c r="E189">
         <v>4</v>
@@ -5830,7 +5830,7 @@
         </is>
       </c>
       <c r="D190">
-        <v>4.04147835320126</v>
+        <v>1.43748052419723</v>
       </c>
       <c r="E190">
         <v>4</v>
@@ -5853,7 +5853,7 @@
         </is>
       </c>
       <c r="D191">
-        <v>0.484737198249527</v>
+        <v>0.742391944659155</v>
       </c>
       <c r="E191">
         <v>4</v>
@@ -5876,7 +5876,7 @@
         </is>
       </c>
       <c r="D192">
-        <v>0.747119074194129</v>
+        <v>0.814475691267739</v>
       </c>
       <c r="E192">
         <v>4</v>
@@ -5899,7 +5899,7 @@
         </is>
       </c>
       <c r="D193">
-        <v>0.838541566514971</v>
+        <v>0.841795960380876</v>
       </c>
       <c r="E193">
         <v>4</v>
@@ -5922,7 +5922,7 @@
         </is>
       </c>
       <c r="D194">
-        <v>0.750479061093666</v>
+        <v>0.578688557247906</v>
       </c>
       <c r="E194">
         <v>4</v>
@@ -5945,7 +5945,7 @@
         </is>
       </c>
       <c r="D195">
-        <v>1.16772791474266</v>
+        <v>0.741259062631576</v>
       </c>
       <c r="E195">
         <v>4</v>
@@ -5968,7 +5968,7 @@
         </is>
       </c>
       <c r="D196">
-        <v>3.97979312216402</v>
+        <v>1.82641330187025</v>
       </c>
       <c r="E196">
         <v>4</v>
@@ -5991,7 +5991,7 @@
         </is>
       </c>
       <c r="D197">
-        <v>5.56631368608131</v>
+        <v>3.85860241271531</v>
       </c>
       <c r="E197">
         <v>4</v>
@@ -6014,7 +6014,7 @@
         </is>
       </c>
       <c r="D198">
-        <v>10.3539487507709</v>
+        <v>3.84439347044957</v>
       </c>
       <c r="E198">
         <v>4</v>
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D199">
-        <v>1.43067101170971</v>
+        <v>1.24033899911088</v>
       </c>
       <c r="E199">
         <v>4</v>
@@ -6060,7 +6060,7 @@
         </is>
       </c>
       <c r="D200">
-        <v>0.787261157211053</v>
+        <v>0.656620563685675</v>
       </c>
       <c r="E200">
         <v>4</v>
@@ -6083,7 +6083,7 @@
         </is>
       </c>
       <c r="D201">
-        <v>0.926786346982391</v>
+        <v>0.696752002497001</v>
       </c>
       <c r="E201">
         <v>4</v>
@@ -6106,7 +6106,7 @@
         </is>
       </c>
       <c r="D202">
-        <v>0.448468458035717</v>
+        <v>0.351896655383807</v>
       </c>
       <c r="E202">
         <v>4</v>
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="D203">
-        <v>0.696485673608879</v>
+        <v>0.432104188236176</v>
       </c>
       <c r="E203">
         <v>4</v>
@@ -6152,7 +6152,7 @@
         </is>
       </c>
       <c r="D204">
-        <v>1.90593383619445</v>
+        <v>0.66593013372301</v>
       </c>
       <c r="E204">
         <v>4</v>
@@ -6175,7 +6175,7 @@
         </is>
       </c>
       <c r="D205">
-        <v>2.44933384008611</v>
+        <v>1.24634191001812</v>
       </c>
       <c r="E205">
         <v>4</v>
@@ -6198,7 +6198,7 @@
         </is>
       </c>
       <c r="D206">
-        <v>5.09069448122856</v>
+        <v>1.25851815296031</v>
       </c>
       <c r="E206">
         <v>4</v>
@@ -6221,7 +6221,7 @@
         </is>
       </c>
       <c r="D207">
-        <v>0.465735620123992</v>
+        <v>0.409224278991971</v>
       </c>
       <c r="E207">
         <v>4</v>
@@ -6244,7 +6244,7 @@
         </is>
       </c>
       <c r="D208">
-        <v>0.455614703991474</v>
+        <v>0.368480470890821</v>
       </c>
       <c r="E208">
         <v>4</v>
@@ -6267,7 +6267,7 @@
         </is>
       </c>
       <c r="D209">
-        <v>0.532292316063163</v>
+        <v>0.398977579007388</v>
       </c>
       <c r="E209">
         <v>4</v>
@@ -6290,7 +6290,7 @@
         </is>
       </c>
       <c r="D210">
-        <v>0.686583015020704</v>
+        <v>0.724117949740903</v>
       </c>
       <c r="E210">
         <v>4</v>
@@ -6313,7 +6313,7 @@
         </is>
       </c>
       <c r="D211">
-        <v>0.884983672711646</v>
+        <v>0.809428074712731</v>
       </c>
       <c r="E211">
         <v>4</v>
@@ -6336,7 +6336,7 @@
         </is>
       </c>
       <c r="D212">
-        <v>2.16373351816136</v>
+        <v>1.20757232573308</v>
       </c>
       <c r="E212">
         <v>4</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="D213">
-        <v>2.5980637828022</v>
+        <v>2.32563736996383</v>
       </c>
       <c r="E213">
         <v>4</v>
@@ -6382,7 +6382,7 @@
         </is>
       </c>
       <c r="D214">
-        <v>3.17434839874017</v>
+        <v>1.88306253863992</v>
       </c>
       <c r="E214">
         <v>4</v>
@@ -6405,7 +6405,7 @@
         </is>
       </c>
       <c r="D215">
-        <v>0.618601720561152</v>
+        <v>0.788841622154112</v>
       </c>
       <c r="E215">
         <v>4</v>
@@ -6428,7 +6428,7 @@
         </is>
       </c>
       <c r="D216">
-        <v>0.690101966631494</v>
+        <v>0.803962795671786</v>
       </c>
       <c r="E216">
         <v>4</v>
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="D217">
-        <v>0.776736985845947</v>
+        <v>0.820247299953307</v>
       </c>
       <c r="E217">
         <v>4</v>
@@ -6474,7 +6474,7 @@
         </is>
       </c>
       <c r="D218">
-        <v>0.875815947979951</v>
+        <v>0.768980796099164</v>
       </c>
       <c r="E218">
         <v>4</v>
@@ -6497,7 +6497,7 @@
         </is>
       </c>
       <c r="D219">
-        <v>1.24462657439414</v>
+        <v>0.88810776341147</v>
       </c>
       <c r="E219">
         <v>4</v>
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="D220">
-        <v>3.3791707513548</v>
+        <v>1.51262371354186</v>
       </c>
       <c r="E220">
         <v>4</v>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="D221">
-        <v>5.49285792702561</v>
+        <v>3.80758733055131</v>
       </c>
       <c r="E221">
         <v>4</v>
@@ -6566,7 +6566,7 @@
         </is>
       </c>
       <c r="D222">
-        <v>7.8012070243111</v>
+        <v>2.23778237412676</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -6589,7 +6589,7 @@
         </is>
       </c>
       <c r="D223">
-        <v>1.56657588355138</v>
+        <v>1.63984506260052</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -6612,7 +6612,7 @@
         </is>
       </c>
       <c r="D224">
-        <v>0.926762447094029</v>
+        <v>0.815532038410042</v>
       </c>
       <c r="E224">
         <v>4</v>
@@ -6635,7 +6635,7 @@
         </is>
       </c>
       <c r="D225">
-        <v>1.04557741468882</v>
+        <v>0.906784364581086</v>
       </c>
       <c r="E225">
         <v>4</v>
@@ -6658,7 +6658,7 @@
         </is>
       </c>
       <c r="D226">
-        <v>0.637106676442478</v>
+        <v>0.683652729258554</v>
       </c>
       <c r="E226">
         <v>4</v>
@@ -6681,7 +6681,7 @@
         </is>
       </c>
       <c r="D227">
-        <v>0.835826247357786</v>
+        <v>0.828856771031316</v>
       </c>
       <c r="E227">
         <v>4</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="D228">
-        <v>2.01439317048966</v>
+        <v>1.35958165505291</v>
       </c>
       <c r="E228">
         <v>4</v>
@@ -6727,7 +6727,7 @@
         </is>
       </c>
       <c r="D229">
-        <v>2.93319424634178</v>
+        <v>3.81028743448662</v>
       </c>
       <c r="E229">
         <v>4</v>
@@ -6750,7 +6750,7 @@
         </is>
       </c>
       <c r="D230">
-        <v>2.98028791873799</v>
+        <v>2.59942358912431</v>
       </c>
       <c r="E230">
         <v>4</v>
@@ -6773,7 +6773,7 @@
         </is>
       </c>
       <c r="D231">
-        <v>0.901284975197852</v>
+        <v>1.08095250968542</v>
       </c>
       <c r="E231">
         <v>4</v>
@@ -6796,7 +6796,7 @@
         </is>
       </c>
       <c r="D232">
-        <v>0.608147039952831</v>
+        <v>0.692435945861428</v>
       </c>
       <c r="E232">
         <v>4</v>
@@ -6819,7 +6819,7 @@
         </is>
       </c>
       <c r="D233">
-        <v>0.735219871073031</v>
+        <v>0.799238947607361</v>
       </c>
       <c r="E233">
         <v>4</v>
@@ -6842,7 +6842,7 @@
         </is>
       </c>
       <c r="D234">
-        <v>0.605948235674677</v>
+        <v>0.728574460152149</v>
       </c>
       <c r="E234">
         <v>4</v>
@@ -6865,7 +6865,7 @@
         </is>
       </c>
       <c r="D235">
-        <v>0.633671567164241</v>
+        <v>0.796345105517848</v>
       </c>
       <c r="E235">
         <v>4</v>
@@ -6888,7 +6888,7 @@
         </is>
       </c>
       <c r="D236">
-        <v>1.65166199842053</v>
+        <v>1.55347950747521</v>
       </c>
       <c r="E236">
         <v>4</v>
@@ -6911,7 +6911,7 @@
         </is>
       </c>
       <c r="D237">
-        <v>2.80156428010859</v>
+        <v>1.94667111969289</v>
       </c>
       <c r="E237">
         <v>4</v>
@@ -6934,7 +6934,7 @@
         </is>
       </c>
       <c r="D238">
-        <v>2.4247068635029</v>
+        <v>3.47113821139223</v>
       </c>
       <c r="E238">
         <v>4</v>
@@ -6957,7 +6957,7 @@
         </is>
       </c>
       <c r="D239">
-        <v>0.777819021135322</v>
+        <v>1.21615633045255</v>
       </c>
       <c r="E239">
         <v>4</v>
@@ -6980,7 +6980,7 @@
         </is>
       </c>
       <c r="D240">
-        <v>0.594840387160502</v>
+        <v>0.777994326515585</v>
       </c>
       <c r="E240">
         <v>4</v>
@@ -7003,7 +7003,7 @@
         </is>
       </c>
       <c r="D241">
-        <v>0.679091271111746</v>
+        <v>0.869490672809403</v>
       </c>
       <c r="E241">
         <v>4</v>
@@ -7765,7 +7765,7 @@
         </is>
       </c>
       <c r="C50">
-        <v>0.974358974358974</v>
+        <v>0.985903715846778</v>
       </c>
     </row>
     <row r="51">
@@ -7780,7 +7780,7 @@
         </is>
       </c>
       <c r="C51">
-        <v>0.888888888888889</v>
+        <v>1.24936001572547</v>
       </c>
     </row>
     <row r="52">
@@ -7795,7 +7795,7 @@
         </is>
       </c>
       <c r="C52">
-        <v>1.24786324786325</v>
+        <v>1.22708722724854</v>
       </c>
     </row>
     <row r="53">
@@ -7810,7 +7810,7 @@
         </is>
       </c>
       <c r="C53">
-        <v>0.752136752136752</v>
+        <v>0.667090094939504</v>
       </c>
     </row>
     <row r="54">
@@ -7825,7 +7825,7 @@
         </is>
       </c>
       <c r="C54">
-        <v>0.94017094017094</v>
+        <v>0.893950429967941</v>
       </c>
     </row>
     <row r="55">
@@ -7840,7 +7840,7 @@
         </is>
       </c>
       <c r="C55">
-        <v>0.905982905982906</v>
+        <v>0.915508381530888</v>
       </c>
     </row>
     <row r="56">
@@ -7855,7 +7855,7 @@
         </is>
       </c>
       <c r="C56">
-        <v>1.35042735042735</v>
+        <v>0.900862420060052</v>
       </c>
     </row>
     <row r="57">
@@ -7870,7 +7870,7 @@
         </is>
       </c>
       <c r="C57">
-        <v>0.94017094017094</v>
+        <v>1.16023771468083</v>
       </c>
     </row>
   </sheetData>
@@ -9006,7 +9006,7 @@
         <v>0.49367581112711</v>
       </c>
       <c r="F2">
-        <v>0.1171875</v>
+        <v>0.078125</v>
       </c>
       <c r="G2">
         <v>3</v>
@@ -9062,7 +9062,7 @@
         <v>0.520315052625641</v>
       </c>
       <c r="F4">
-        <v>0.84765625</v>
+        <v>0.6015625</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -9106,25 +9106,25 @@
         </is>
       </c>
       <c r="B6">
-        <v>0.175078468060665</v>
+        <v>0.271723506555857</v>
       </c>
       <c r="C6">
-        <v>0.188356671520292</v>
+        <v>0.299497614693099</v>
       </c>
       <c r="D6">
-        <v>-0.0185993518770528</v>
+        <v>0.0524822999213043</v>
       </c>
       <c r="E6">
-        <v>0.385980377372675</v>
+        <v>0.535271161066248</v>
       </c>
       <c r="F6">
-        <v>0.015625</v>
+        <v>0.30078125</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>0.111006211187289</v>
+        <v>0.126707356693466</v>
       </c>
     </row>
   </sheetData>
@@ -9276,7 +9276,7 @@
         </is>
       </c>
       <c r="C8">
-        <v>0.361531641289371</v>
+        <v>0.426951411329971</v>
       </c>
       <c r="D8">
         <v>7</v>
@@ -9294,7 +9294,7 @@
         </is>
       </c>
       <c r="C9">
-        <v>0.0160988411769178</v>
+        <v>0.142713528925734</v>
       </c>
       <c r="D9">
         <v>7</v>
@@ -9354,16 +9354,16 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>0.207955274412409</v>
+        <v>0.34771674396399</v>
       </c>
       <c r="D2">
-        <v>4.76742011526803</v>
+        <v>2.3071138880091</v>
       </c>
       <c r="E2">
-        <v>-15.049734535765</v>
+        <v>3.2321799056425</v>
       </c>
       <c r="F2">
-        <v>7.29579758588911</v>
+        <v>5.24862264844391</v>
       </c>
       <c r="G2">
         <v>0.133003150692219</v>
@@ -9379,16 +9379,16 @@
         <v>8</v>
       </c>
       <c r="C3">
-        <v>0.191213433578383</v>
+        <v>0.281138446356604</v>
       </c>
       <c r="D3">
-        <v>4.70219850653354</v>
+        <v>2.46649319213784</v>
       </c>
       <c r="E3">
-        <v>-14.1007333144717</v>
+        <v>-1.19712562736273</v>
       </c>
       <c r="F3">
-        <v>6.93589275254453</v>
+        <v>5.07111691795643</v>
       </c>
       <c r="G3">
         <v>0.133003150692219</v>
@@ -9404,16 +9404,16 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>0.186864101026427</v>
+        <v>0.224853339336294</v>
       </c>
       <c r="D4">
-        <v>4.47763220193772</v>
+        <v>2.35760209926459</v>
       </c>
       <c r="E4">
-        <v>-15.1246245426118</v>
+        <v>-4.02765516467641</v>
       </c>
       <c r="F4">
-        <v>6.50667709677349</v>
+        <v>4.75236977247757</v>
       </c>
       <c r="G4">
         <v>0.133003150692219</v>
@@ -9429,16 +9429,16 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <v>0.172243874621758</v>
+        <v>0.242919556912903</v>
       </c>
       <c r="D5">
-        <v>4.31555148793795</v>
+        <v>2.26865569215702</v>
       </c>
       <c r="E5">
-        <v>-14.5888178038692</v>
+        <v>-3.22322674146571</v>
       </c>
       <c r="F5">
-        <v>6.22223451613308</v>
+        <v>4.53768027507191</v>
       </c>
       <c r="G5">
         <v>0.133003150692219</v>
@@ -9563,14 +9563,14 @@
         </is>
       </c>
       <c r="E3">
-        <v>0.19265840974003</v>
+        <v>0.282745827922781</v>
       </c>
       <c r="F3"/>
       <c r="G3">
-        <v>4.70219850653354</v>
+        <v>2.46649319213784</v>
       </c>
       <c r="H3">
-        <v>-14.8067266070864</v>
+        <v>-1.25301726373385</v>
       </c>
       <c r="I3">
         <v>0.133003150692219</v>
@@ -9633,14 +9633,14 @@
         </is>
       </c>
       <c r="E5">
-        <v>0.121069837168429</v>
+        <v>0.195943228598931</v>
       </c>
       <c r="F5"/>
       <c r="G5">
-        <v>4.70219850653354</v>
+        <v>2.46649319213784</v>
       </c>
       <c r="H5">
-        <v>-17.0114468896617</v>
+        <v>-2.97066653857816</v>
       </c>
       <c r="I5">
         <v>0.0684112247307324</v>
@@ -9703,14 +9703,14 @@
         </is>
       </c>
       <c r="E7">
-        <v>0.200241033555834</v>
+        <v>0.32588656016322</v>
       </c>
       <c r="F7"/>
       <c r="G7">
-        <v>4.70219850653354</v>
+        <v>2.46649319213784</v>
       </c>
       <c r="H7">
-        <v>-8.85478251311323</v>
+        <v>4.30569266744704</v>
       </c>
       <c r="I7">
         <v>0.0814422567890167</v>
@@ -9773,14 +9773,14 @@
         </is>
       </c>
       <c r="E9">
-        <v>0.199096010154098</v>
+        <v>0.154082622926873</v>
       </c>
       <c r="F9"/>
       <c r="G9">
-        <v>4.70219850653354</v>
+        <v>2.46649319213784</v>
       </c>
       <c r="H9">
-        <v>-4.36792322961975</v>
+        <v>-0.981396779439282</v>
       </c>
       <c r="I9">
         <v>-0.0304196852696619</v>
@@ -9818,10 +9818,15 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>raw_status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>score</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>evidence</t>
         </is>
@@ -9843,13 +9848,18 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>proxy-supported</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>implemented_first_pass</t>
         </is>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>0.332605705883613</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>sensory-transmodal, associative, thalamic-gateway, and hierarchy-flattening FC proxies</t>
         </is>
@@ -9871,15 +9881,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>implemented_proxy_control_energy</t>
         </is>
       </c>
-      <c r="E3">
-        <v>0.175078468060665</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>finite-horizon control energy with receptor, hierarchy, transmodal, random, and degree-control profiles</t>
+      <c r="F3">
+        <v>0.271723506555857</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>finite-horizon lower transition/control-energy proxy; receptor-specific placement remains unsupported without structural/PET/spatial-null gates</t>
         </is>
       </c>
     </row>
@@ -9899,13 +9914,18 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>implemented_first_pass</t>
         </is>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>0.150618725276116</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>integration, segregation, graph modularity, participation, dynamic-FC variance, and trajectory-step proxies</t>
         </is>
@@ -9927,13 +9947,18 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>implemented_first_pass</t>
         </is>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>0.148906094111187</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>state occupancy, transition entropy, transition rate, dwell/barrier, and step-distance proxies</t>
         </is>
@@ -9955,13 +9980,18 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>implemented_negative_control_baseline</t>
         </is>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>-0.0740636981753378</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>leave-one-subject-out one-step RMSE change; retained as a predictive baseline, not control-energy evidence</t>
         </is>
@@ -10421,7 +10451,7 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>4.70219850653354</v>
+        <v>2.46649319213784</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -10447,7 +10477,7 @@
         </is>
       </c>
       <c r="L6">
-        <v>0.375766048442555</v>
+        <v>0.190760953510083</v>
       </c>
     </row>
     <row r="7">
@@ -10475,7 +10505,7 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>-15.0826173674297</v>
+        <v>-1.84424642546406</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -10501,7 +10531,7 @@
         </is>
       </c>
       <c r="L7">
-        <v>-0.863310282113102</v>
+        <v>-0.1289201435325</v>
       </c>
     </row>
     <row r="8">
@@ -10517,7 +10547,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>not_available_current_8_module_proxy</t>
+          <t>not_available_current_proxy_without_striatal_parcel</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -10539,7 +10569,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Do not claim striatal support from the current Harvard-Oxford 8-module proxy.</t>
+          <t>Do not claim striatal support from cortical-only or current 8-module proxy rows.</t>
         </is>
       </c>
       <c r="J8">
@@ -10584,17 +10614,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C hierarchy/routing is currently the strongest implemented LSD mechanism layer.</t>
+          <t>C is the provisional leading macro-dynamic proxy under the current cached ds003059 analysis, pending motion/confound control and atlas-level replication.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>supported_first_pass</t>
+          <t>proxy-supported</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bootstrap rank-1 fraction=0.848.</t>
+          <t>Bootstrap rank-1 fraction=0.602.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -10611,12 +10641,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>supported_proxy</t>
+          <t>proxy-supported</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Default-horizon receptor transition-energy reduction=4.702%.</t>
+          <t>Default-horizon receptor transition-energy reduction=2.466%.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -10633,12 +10663,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>not_supported_yet</t>
+          <t>unsupported</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Receptor-vs-random energy reduction=-15.083%.</t>
+          <t>Receptor-vs-random energy reduction=-1.844%.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -10655,7 +10685,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>directionally_aligned</t>
+          <t>proxy-supported</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -10677,12 +10707,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>not_testable_current_proxy</t>
+          <t>future</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>not_available_current_8_module_proxy</t>
+          <t>not_available_current_proxy_without_striatal_parcel</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -10694,12 +10724,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B DMDc is the main control-theory result.</t>
+          <t>Rejected candidate: B DMDc as the main control-theory result.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>reject_as_main_claim</t>
+          <t>unsupported</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -21460,25 +21490,25 @@
         </is>
       </c>
       <c r="B2">
-        <v>4.70219850653354</v>
+        <v>2.46649319213784</v>
       </c>
       <c r="C2">
-        <v>12.5136332194535</v>
+        <v>12.9297591920847</v>
       </c>
       <c r="D2">
-        <v>0.375766048442555</v>
+        <v>0.190760953510083</v>
       </c>
       <c r="E2">
-        <v>0.375766048442555</v>
+        <v>0.190760953510083</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>0.633333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="H2">
-        <v>0.100244211032987</v>
+        <v>0.572232224047184</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -21498,25 +21528,25 @@
         </is>
       </c>
       <c r="B3">
-        <v>6.93589275254453</v>
+        <v>5.07111691795643</v>
       </c>
       <c r="C3">
-        <v>9.57709062623694</v>
+        <v>9.03278708436657</v>
       </c>
       <c r="D3">
-        <v>0.724217095068861</v>
+        <v>0.561412205401501</v>
       </c>
       <c r="E3">
-        <v>0.724217095068861</v>
+        <v>0.561412205401501</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>0.766666666666667</v>
+        <v>0.7</v>
       </c>
       <c r="H3">
-        <v>0.0026114396750927</v>
+        <v>0.0213869726285338</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -21536,25 +21566,25 @@
         </is>
       </c>
       <c r="B4">
-        <v>-34.3869884708404</v>
+        <v>-18.8548996710124</v>
       </c>
       <c r="C4">
-        <v>23.5868587891858</v>
+        <v>17.3029344949926</v>
       </c>
       <c r="D4">
-        <v>-1.45788757961303</v>
+        <v>-1.08969375549962</v>
       </c>
       <c r="E4">
-        <v>-1.45788757961303</v>
+        <v>-1.08969375549962</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>0.999995784834027</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -21574,25 +21604,25 @@
         </is>
       </c>
       <c r="B5">
-        <v>-15.0826173674297</v>
+        <v>-1.84424642546406</v>
       </c>
       <c r="C5">
-        <v>17.47067963851</v>
+        <v>14.3053395298085</v>
       </c>
       <c r="D5">
-        <v>-0.863310282113102</v>
+        <v>-0.1289201435325</v>
       </c>
       <c r="E5">
-        <v>-0.863310282113102</v>
+        <v>-0.1289201435325</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="H5">
-        <v>0.991937599144876</v>
+        <v>0.180797304026783</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -21612,16 +21642,16 @@
         </is>
       </c>
       <c r="B6">
-        <v>-300.469563048223</v>
+        <v>-136.409009912745</v>
       </c>
       <c r="C6">
-        <v>130.810742371499</v>
+        <v>94.6131394859698</v>
       </c>
       <c r="D6">
-        <v>-2.29697926638852</v>
+        <v>-1.44175545440994</v>
       </c>
       <c r="E6">
-        <v>-2.29697926638852</v>
+        <v>-1.44175545440994</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -21650,16 +21680,16 @@
         </is>
       </c>
       <c r="B7">
-        <v>-674.315980973865</v>
+        <v>-288.488440982514</v>
       </c>
       <c r="C7">
-        <v>331.412656625716</v>
+        <v>191.246799107827</v>
       </c>
       <c r="D7">
-        <v>-2.0346717830255</v>
+        <v>-1.50846153937385</v>
       </c>
       <c r="E7">
-        <v>-2.0346717830255</v>
+        <v>-1.50846153937385</v>
       </c>
       <c r="F7">
         <v>1</v>

</xml_diff>